<commit_message>
Group overview of all 35 images, and the QC list of the 27 new ones
group-overview regenerated: results/group_overview.csv and .xlsx, one row
per image of all four groups (WT rows unchanged). group-qc run:
results/group_qc.csv, per image of WT_HP, Hyp_RD and Hyp_HP, against the
WT range of 11 to 19 lacunae. 19 of the 27 are outside it: 16 of the 18
Hyp images (24 to 50 lacunae) and 3 of WT_HP (8, 10 and 21). No
statistic and no comparison between groups.

group-qc gains -w (default 8): the lacuna stage of each image is rerun in
its own process, the same work as before only in parallel; on WT it gives
exactly the sequential result. The run took 68 minutes, most of it one
image, 701_z19.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/group_overview.xlsx
+++ b/results/group_overview.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -753,6 +753,978 @@
       </c>
       <c r="J9" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>872_wt_hp_z03</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>326.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.02771351</v>
+      </c>
+      <c r="H10" t="n">
+        <v>27705</v>
+      </c>
+      <c r="I10" t="n">
+        <v>11000</v>
+      </c>
+      <c r="J10" t="n">
+        <v>7.2111</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>872_wt_hp_z04</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>21</v>
+      </c>
+      <c r="D11" t="n">
+        <v>18</v>
+      </c>
+      <c r="E11" t="n">
+        <v>11.9444</v>
+      </c>
+      <c r="F11" t="n">
+        <v>497.6667</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.03842741</v>
+      </c>
+      <c r="H11" t="n">
+        <v>38673</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3314</v>
+      </c>
+      <c r="J11" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>872_wt_hp_z06</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D12" t="n">
+        <v>14</v>
+      </c>
+      <c r="E12" t="n">
+        <v>10.2857</v>
+      </c>
+      <c r="F12" t="n">
+        <v>435.0714</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.03813472</v>
+      </c>
+      <c r="H12" t="n">
+        <v>39179</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4957</v>
+      </c>
+      <c r="J12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>876_z76c1-2</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8.7143</v>
+      </c>
+      <c r="F13" t="n">
+        <v>568.1429000000001</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.06422000999999999</v>
+      </c>
+      <c r="H13" t="n">
+        <v>66385</v>
+      </c>
+      <c r="I13" t="n">
+        <v>20047</v>
+      </c>
+      <c r="J13" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>876_z82c1-2</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" t="n">
+        <v>9.333299999999999</v>
+      </c>
+      <c r="F14" t="n">
+        <v>544</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.06998144000000001</v>
+      </c>
+      <c r="H14" t="n">
+        <v>72148</v>
+      </c>
+      <c r="I14" t="n">
+        <v>15814</v>
+      </c>
+      <c r="J14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>876_z89c1-2</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D15" t="n">
+        <v>11</v>
+      </c>
+      <c r="E15" t="n">
+        <v>11.3636</v>
+      </c>
+      <c r="F15" t="n">
+        <v>669.9091</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.07920204</v>
+      </c>
+      <c r="H15" t="n">
+        <v>80679</v>
+      </c>
+      <c r="I15" t="n">
+        <v>11140</v>
+      </c>
+      <c r="J15" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>877_wt_z073c1-2</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>14</v>
+      </c>
+      <c r="D16" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" t="n">
+        <v>9.333299999999999</v>
+      </c>
+      <c r="F16" t="n">
+        <v>362.0833</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.03100654</v>
+      </c>
+      <c r="H16" t="n">
+        <v>31505</v>
+      </c>
+      <c r="I16" t="n">
+        <v>14241</v>
+      </c>
+      <c r="J16" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>877_wt_z081c1-2</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="F17" t="n">
+        <v>309</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.03195255</v>
+      </c>
+      <c r="H17" t="n">
+        <v>32368</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12675</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WT_HP</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>877_wt_z087c1-2</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>11</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" t="n">
+        <v>12.7143</v>
+      </c>
+      <c r="F18" t="n">
+        <v>411.2857</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.03064417</v>
+      </c>
+      <c r="H18" t="n">
+        <v>31010</v>
+      </c>
+      <c r="I18" t="n">
+        <v>14531</v>
+      </c>
+      <c r="J18" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>535_z13c1-2</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>32</v>
+      </c>
+      <c r="D19" t="n">
+        <v>27</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6.8519</v>
+      </c>
+      <c r="F19" t="n">
+        <v>218</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.02090037</v>
+      </c>
+      <c r="H19" t="n">
+        <v>20589</v>
+      </c>
+      <c r="I19" t="n">
+        <v>8617</v>
+      </c>
+      <c r="J19" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>535_z20c1-2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>30</v>
+      </c>
+      <c r="D20" t="n">
+        <v>22</v>
+      </c>
+      <c r="E20" t="n">
+        <v>7.5909</v>
+      </c>
+      <c r="F20" t="n">
+        <v>244.3636</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.02245659</v>
+      </c>
+      <c r="H20" t="n">
+        <v>21893</v>
+      </c>
+      <c r="I20" t="n">
+        <v>9303</v>
+      </c>
+      <c r="J20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>535_z27c1-2</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>31</v>
+      </c>
+      <c r="D21" t="n">
+        <v>27</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6.2593</v>
+      </c>
+      <c r="F21" t="n">
+        <v>203.1852</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.02474458</v>
+      </c>
+      <c r="H21" t="n">
+        <v>24026</v>
+      </c>
+      <c r="I21" t="n">
+        <v>11669</v>
+      </c>
+      <c r="J21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>536-63x_Hyp_RD_z03c1-2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>24</v>
+      </c>
+      <c r="D22" t="n">
+        <v>20</v>
+      </c>
+      <c r="E22" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>277.95</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.02197568</v>
+      </c>
+      <c r="H22" t="n">
+        <v>21555</v>
+      </c>
+      <c r="I22" t="n">
+        <v>10731</v>
+      </c>
+      <c r="J22" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>536-63x_Hyp_RD_z08c1-2</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>29</v>
+      </c>
+      <c r="D23" t="n">
+        <v>25</v>
+      </c>
+      <c r="E23" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="F23" t="n">
+        <v>279.48</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.02691272</v>
+      </c>
+      <c r="H23" t="n">
+        <v>25440</v>
+      </c>
+      <c r="I23" t="n">
+        <v>8426</v>
+      </c>
+      <c r="J23" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>536-63x_Hyp_RD_z15c1-2</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>15</v>
+      </c>
+      <c r="D24" t="n">
+        <v>13</v>
+      </c>
+      <c r="E24" t="n">
+        <v>8.0769</v>
+      </c>
+      <c r="F24" t="n">
+        <v>262.3077</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.02605206</v>
+      </c>
+      <c r="H24" t="n">
+        <v>25413</v>
+      </c>
+      <c r="I24" t="n">
+        <v>11875</v>
+      </c>
+      <c r="J24" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>I534_z11c1-2</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>42</v>
+      </c>
+      <c r="D25" t="n">
+        <v>33</v>
+      </c>
+      <c r="E25" t="n">
+        <v>9.4848</v>
+      </c>
+      <c r="F25" t="n">
+        <v>257.1212</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.0285107</v>
+      </c>
+      <c r="H25" t="n">
+        <v>25190</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4533</v>
+      </c>
+      <c r="J25" t="n">
+        <v>8.2462</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>I534_z19c1-2</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>37</v>
+      </c>
+      <c r="D26" t="n">
+        <v>29</v>
+      </c>
+      <c r="E26" t="n">
+        <v>9.793100000000001</v>
+      </c>
+      <c r="F26" t="n">
+        <v>257.1034</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.02658338</v>
+      </c>
+      <c r="H26" t="n">
+        <v>23531</v>
+      </c>
+      <c r="I26" t="n">
+        <v>7073</v>
+      </c>
+      <c r="J26" t="n">
+        <v>8.2462</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hyp_RD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>I534_z25c1-2</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>37</v>
+      </c>
+      <c r="D27" t="n">
+        <v>26</v>
+      </c>
+      <c r="E27" t="n">
+        <v>6.2308</v>
+      </c>
+      <c r="F27" t="n">
+        <v>212.6923</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.02567676</v>
+      </c>
+      <c r="H27" t="n">
+        <v>23402</v>
+      </c>
+      <c r="I27" t="n">
+        <v>7454</v>
+      </c>
+      <c r="J27" t="n">
+        <v>8.2462</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>548_hyp_HP_z08c1-2</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>29</v>
+      </c>
+      <c r="D28" t="n">
+        <v>24</v>
+      </c>
+      <c r="E28" t="n">
+        <v>8.666700000000001</v>
+      </c>
+      <c r="F28" t="n">
+        <v>263.25</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.02803206</v>
+      </c>
+      <c r="H28" t="n">
+        <v>27514</v>
+      </c>
+      <c r="I28" t="n">
+        <v>12303</v>
+      </c>
+      <c r="J28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>548_hyp_HP_z14c1-2</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>29</v>
+      </c>
+      <c r="D29" t="n">
+        <v>21</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8.4762</v>
+      </c>
+      <c r="F29" t="n">
+        <v>273.6667</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.02801933</v>
+      </c>
+      <c r="H29" t="n">
+        <v>27424</v>
+      </c>
+      <c r="I29" t="n">
+        <v>8607</v>
+      </c>
+      <c r="J29" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>548_hyp_HP_z20c1-2</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>32</v>
+      </c>
+      <c r="D30" t="n">
+        <v>25</v>
+      </c>
+      <c r="E30" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="F30" t="n">
+        <v>228.16</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.02540235</v>
+      </c>
+      <c r="H30" t="n">
+        <v>25128</v>
+      </c>
+      <c r="I30" t="n">
+        <v>10547</v>
+      </c>
+      <c r="J30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>699_HYP_HP_z11c1-2</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>30</v>
+      </c>
+      <c r="D31" t="n">
+        <v>25</v>
+      </c>
+      <c r="E31" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="F31" t="n">
+        <v>295.32</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.02274098</v>
+      </c>
+      <c r="H31" t="n">
+        <v>21874</v>
+      </c>
+      <c r="I31" t="n">
+        <v>5852</v>
+      </c>
+      <c r="J31" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>699_HYP_HP_z20c1-2</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>25</v>
+      </c>
+      <c r="D32" t="n">
+        <v>21</v>
+      </c>
+      <c r="E32" t="n">
+        <v>5.6667</v>
+      </c>
+      <c r="F32" t="n">
+        <v>197.2381</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.01784047</v>
+      </c>
+      <c r="H32" t="n">
+        <v>17690</v>
+      </c>
+      <c r="I32" t="n">
+        <v>8209</v>
+      </c>
+      <c r="J32" t="n">
+        <v>7.2111</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>699_HYP_HP_z25c1-2</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>17</v>
+      </c>
+      <c r="D33" t="n">
+        <v>13</v>
+      </c>
+      <c r="E33" t="n">
+        <v>4.7692</v>
+      </c>
+      <c r="F33" t="n">
+        <v>214</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.01669379</v>
+      </c>
+      <c r="H33" t="n">
+        <v>16779</v>
+      </c>
+      <c r="I33" t="n">
+        <v>9250</v>
+      </c>
+      <c r="J33" t="n">
+        <v>7.2111</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>701_z19c1-2</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>50</v>
+      </c>
+      <c r="D34" t="n">
+        <v>39</v>
+      </c>
+      <c r="E34" t="n">
+        <v>8.8718</v>
+      </c>
+      <c r="F34" t="n">
+        <v>295.0513</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.04283569</v>
+      </c>
+      <c r="H34" t="n">
+        <v>36760</v>
+      </c>
+      <c r="I34" t="n">
+        <v>8290</v>
+      </c>
+      <c r="J34" t="n">
+        <v>7.2111</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>701_z26c1-2</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>45</v>
+      </c>
+      <c r="D35" t="n">
+        <v>33</v>
+      </c>
+      <c r="E35" t="n">
+        <v>7.6364</v>
+      </c>
+      <c r="F35" t="n">
+        <v>286.0606</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.04889893</v>
+      </c>
+      <c r="H35" t="n">
+        <v>43791</v>
+      </c>
+      <c r="I35" t="n">
+        <v>15082</v>
+      </c>
+      <c r="J35" t="n">
+        <v>6.3246</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hyp_HP</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>701_z36c1-2</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>30</v>
+      </c>
+      <c r="D36" t="n">
+        <v>18</v>
+      </c>
+      <c r="E36" t="n">
+        <v>8.1111</v>
+      </c>
+      <c r="F36" t="n">
+        <v>346.4444</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.06000947</v>
+      </c>
+      <c r="H36" t="n">
+        <v>57414</v>
+      </c>
+      <c r="I36" t="n">
+        <v>21435</v>
+      </c>
+      <c r="J36" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -766,7 +1738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -776,27 +1748,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>WT_HP: no results. all 9 source files were skipped by the import rule (JPEG content; JPEG content, although it is named .tif).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hyp_RD: no results. all 9 source files were skipped by the import rule (JPEG content).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Hyp_HP: no results. all 9 source files were skipped by the import rule (JPEG content).</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>